<commit_message>
formulaire v2 simplifié + registre chantiers
</commit_message>
<xml_diff>
--- a/field/hanoi_noise_form_v2.xlsx
+++ b/field/hanoi_noise_form_v2.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,11 +469,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>constraint_message</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>relevant</t>
         </is>
       </c>
     </row>
@@ -494,7 +489,6 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -513,7 +507,6 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -542,7 +535,6 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -571,7 +563,6 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -600,7 +591,6 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -629,7 +619,6 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -666,7 +655,6 @@
           <t>Value must be between 20 and 120 dB</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -699,7 +687,6 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -728,7 +715,6 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -757,93 +743,82 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>select_one phone_or</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>video_traffic</t>
+          <t>phone_orientation</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Traffic video (15-30 s, phone held HIGH facing the road)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Required during rush hours (07-09h, 17-19h). Second phone measures dB meanwhile.</t>
-        </is>
-      </c>
+          <t>Phone held</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="b">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one mic_dir</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>count_motorbikes</t>
+          <t>mic_to_source</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Motorbikes passing during measurement</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Count during the ~15 s of measurement (estimate if many)</t>
-        </is>
-      </c>
+          <t>Mic relative to the main source</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="b">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 500</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Between 0 and 500</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>count_cars</t>
+          <t>dist_to_source_m</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cars/trucks/buses passing during measurement</t>
+          <t>Estimated distance to the MAIN source (m)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Count during the ~15 s of measurement</t>
+          <t>The dominant source selected in "Main noise category"</t>
         </is>
       </c>
       <c r="E14" t="b">
@@ -852,184 +827,142 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>. &gt;= 0 and . &lt;= 500</t>
+          <t>. &gt;= 0 and . &lt;= 1000</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Between 0 and 500</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>Between 0 and 1000 m</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>select_one source_dir</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>source_direction</t>
+          <t>count_motorbikes</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Direction to the main noise source</t>
+          <t>Motorbikes passing during measurement</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Horizontal = street level; vertical = above/below (construction floor, AC units...)</t>
+          <t>Count during the ~15 s of measurement (estimate if many)</t>
         </is>
       </c>
       <c r="E15" t="b">
         <v>0</v>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 500</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Between 0 and 500</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>dist_to_source_m</t>
+          <t>count_cars</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Estimated distance to the MAIN source (m)</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>The dominant source you selected in "Main noise category"</t>
-        </is>
-      </c>
+          <t>Cars/trucks/buses passing during measurement</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="b">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>. &gt;= 0 and . &lt;= 1000</t>
+          <t>. &gt;= 0 and . &lt;= 500</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Between 0 and 1000 m</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>Between 0 and 500</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>select_one construction</t>
+          <t>video</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>construction_nearby</t>
+          <t>video_traffic</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Construction/demolition site nearby?</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>Traffic video (15-30 s, phone held HIGH facing the road)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Rush hours (07-09h, 17-19h), in pairs: one films, one measures dB</t>
+        </is>
+      </c>
       <c r="E17" t="b">
         <v>0</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>minimal</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>select_one yesno</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>construction_dist_m</t>
+          <t>construction_nearby</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Distance to the construction site (m)</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>Construction/demolition audible from here?</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>If yes and not yet logged, also fill the "Construction sites" form</t>
+        </is>
+      </c>
       <c r="E18" t="b">
         <v>0</v>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 1000</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Between 0 and 1000 m</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>${construction_nearby} != '' and ${construction_nearby} != 'none'</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>construction_note</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Construction site description (optional)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>What is being built/demolished, size, activity level</t>
-        </is>
-      </c>
-      <c r="E19" t="b">
-        <v>0</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>${construction_nearby} != '' and ${construction_nearby} != 'none'</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>minimal</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1042,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1456,102 +1389,136 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>source_dir</t>
+          <t>phone_or</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>horizontal</t>
+          <t>vertical</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Horizontal (street level)</t>
+          <t>Vertical</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>source_dir</t>
+          <t>phone_or</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>vertical</t>
+          <t>horizontal</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Vertical (above or below)</t>
+          <t>Horizontal</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>source_dir</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>towards</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mixed / ambient</t>
+          <t>Pointing towards the source</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>perpendicular</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Perpendicular to the source</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>away</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Yes — construction</t>
+          <t>Back to the source</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>construction</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>demolition</t>
+          <t>above_below</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Yes — demolition/destruction</t>
+          <t>Source above or below</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>yesno</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>yesno</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1556,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026061201</t>
+          <t>2026061202</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tranches distance 0-2 et 2-10
</commit_message>
<xml_diff>
--- a/field/hanoi_noise_form_v2.xlsx
+++ b/field/hanoi_noise_form_v2.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="b">
+      <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="b">
+      <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -585,7 +585,7 @@
           <t>Stand still a few seconds for better accuracy</t>
         </is>
       </c>
-      <c r="E6" t="b">
+      <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -613,7 +613,7 @@
           <t>Record at least 10 s of ambient sound</t>
         </is>
       </c>
-      <c r="E7" t="b">
+      <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -641,7 +641,7 @@
           <t>Read LAeq / average value from the dB app</t>
         </is>
       </c>
-      <c r="E8" t="b">
+      <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -677,7 +677,7 @@
           <t>Dominant sound source</t>
         </is>
       </c>
-      <c r="E9" t="b">
+      <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="b">
+      <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -737,7 +737,7 @@
           <t>Unusual events: horn burst, rain, festival...</t>
         </is>
       </c>
-      <c r="E11" t="b">
+      <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -761,7 +761,7 @@
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="b">
+      <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="b">
+      <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -821,7 +821,7 @@
           <t>The dominant source selected in "Main noise category"</t>
         </is>
       </c>
-      <c r="E14" t="b">
+      <c r="E14" t="n">
         <v>0</v>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -857,7 +857,7 @@
           <t>Count during the ~15 s of measurement (estimate if many)</t>
         </is>
       </c>
-      <c r="E15" t="b">
+      <c r="E15" t="n">
         <v>0</v>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="b">
+      <c r="E16" t="n">
         <v>0</v>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -925,7 +925,7 @@
           <t>Rush hours (07-09h, 17-19h), in pairs: one films, one measures dB</t>
         </is>
       </c>
-      <c r="E17" t="b">
+      <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -953,7 +953,7 @@
           <t>If yes and not yet logged, also fill the "Construction sites" form</t>
         </is>
       </c>
-      <c r="E18" t="b">
+      <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -975,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1321,204 +1321,221 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dist</t>
+          <t>phone_or</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d_0_10</t>
+          <t>vertical</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0-10 m</t>
+          <t>Vertical</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dist</t>
+          <t>phone_or</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d_10_30</t>
+          <t>horizontal</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10-30 m</t>
+          <t>Horizontal</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>dist</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d_30_60</t>
+          <t>towards</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>30-60 m</t>
+          <t>Pointing towards the source</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>dist</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d_60plus</t>
+          <t>perpendicular</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&gt; 60 m / behind building</t>
+          <t>Perpendicular to the source</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>phone_or</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vertical</t>
+          <t>away</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Vertical</t>
+          <t>Back to the source</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>phone_or</t>
+          <t>mic_dir</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>horizontal</t>
+          <t>above_below</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Horizontal</t>
+          <t>Source above or below</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>mic_dir</t>
+          <t>yesno</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>towards</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pointing towards the source</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>mic_dir</t>
+          <t>yesno</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>perpendicular</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Perpendicular to the source</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>mic_dir</t>
+          <t>dist</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>away</t>
+          <t>d_0_2</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Back to the source</t>
+          <t>0-2 m (roadside)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>mic_dir</t>
+          <t>dist</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>above_below</t>
+          <t>d_2_10</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Source above or below</t>
+          <t>2-10 m</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>yesno</t>
+          <t>dist</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>d_10_30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>10-30 m</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>yesno</t>
+          <t>dist</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>d_30_60</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>30-60 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>dist</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>d_60plus</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>&gt; 60 m / behind building</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1573,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026061202</t>
+          <t>2026061203</t>
         </is>
       </c>
     </row>

</xml_diff>